<commit_message>
feat: Implement nursing services mapping and enhance Excel report generation for medical and nursing sections
</commit_message>
<xml_diff>
--- a/backend/api-consulmdregister/storage/app/templates/informe_medico_template.xlsx
+++ b/backend/api-consulmdregister/storage/app/templates/informe_medico_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\CR_Clinik_Reynosa\backend\api-consulmdregister\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8B3B29D-96E5-40D1-A8D3-9899813B9B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38BD2F5-33FF-45D7-8564-1BC06F01079D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SERVICIOS MEDICOS" sheetId="1" r:id="rId1"/>
@@ -1090,23 +1090,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1120,7 +1111,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1174,6 +1174,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1182,12 +1200,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1201,25 +1213,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1228,13 +1231,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1261,9 +1261,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2315,97 +2313,97 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="30"/>
-      <c r="S3" s="30"/>
-      <c r="T3" s="30"/>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="36"/>
+      <c r="V3" s="36"/>
     </row>
     <row r="4" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I4" s="30" t="s">
+      <c r="I4" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="30"/>
-      <c r="T4" s="30"/>
-      <c r="U4" s="30"/>
-      <c r="V4" s="30"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
     </row>
     <row r="5" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I5" s="30" t="s">
+      <c r="I5" s="36" t="s">
         <v>111</v>
       </c>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="36"/>
+      <c r="R5" s="36"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="36"/>
+      <c r="U5" s="36"/>
+      <c r="V5" s="36"/>
     </row>
     <row r="6" spans="2:35" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I6" s="31" t="s">
+      <c r="I6" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="31"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="31"/>
-      <c r="S6" s="31"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="31"/>
-      <c r="V6" s="31"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
+      <c r="S6" s="37"/>
+      <c r="T6" s="37"/>
+      <c r="U6" s="37"/>
+      <c r="V6" s="37"/>
     </row>
     <row r="7" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="K7" s="27" t="s">
+      <c r="K7" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="L7" s="27"/>
-      <c r="M7" s="27"/>
-      <c r="N7" s="27"/>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="27"/>
-      <c r="T7" s="27"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="34"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="34"/>
+      <c r="S7" s="34"/>
+      <c r="T7" s="34"/>
     </row>
     <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="37" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="37"/>
+      <c r="B9" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="28"/>
       <c r="D9" s="4">
         <v>1</v>
       </c>
@@ -2504,10 +2502,10 @@
       </c>
     </row>
     <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="8">
         <v>0</v>
       </c>
@@ -2607,10 +2605,10 @@
       </c>
     </row>
     <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="32"/>
+      <c r="C11" s="27"/>
       <c r="D11" s="8">
         <v>0</v>
       </c>
@@ -2710,10 +2708,10 @@
       </c>
     </row>
     <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="32"/>
+      <c r="C12" s="27"/>
       <c r="D12" s="8">
         <v>0</v>
       </c>
@@ -2813,10 +2811,10 @@
       </c>
     </row>
     <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="C13" s="32"/>
+      <c r="C13" s="27"/>
       <c r="D13" s="8">
         <v>0</v>
       </c>
@@ -2916,10 +2914,10 @@
       </c>
     </row>
     <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="32"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="8">
         <v>0</v>
       </c>
@@ -3019,10 +3017,10 @@
       </c>
     </row>
     <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="32"/>
+      <c r="C15" s="27"/>
       <c r="D15" s="8">
         <v>0</v>
       </c>
@@ -3122,10 +3120,10 @@
       </c>
     </row>
     <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="32"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="8">
         <v>0</v>
       </c>
@@ -3225,10 +3223,10 @@
       </c>
     </row>
     <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="32"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="8">
         <v>0</v>
       </c>
@@ -3328,10 +3326,10 @@
       </c>
     </row>
     <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="32"/>
+      <c r="C18" s="27"/>
       <c r="D18" s="8">
         <v>0</v>
       </c>
@@ -3431,10 +3429,10 @@
       </c>
     </row>
     <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="32"/>
+      <c r="C19" s="27"/>
       <c r="D19" s="8">
         <v>0</v>
       </c>
@@ -3534,10 +3532,10 @@
       </c>
     </row>
     <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="32"/>
+      <c r="C20" s="27"/>
       <c r="D20" s="8">
         <v>0</v>
       </c>
@@ -3637,10 +3635,10 @@
       </c>
     </row>
     <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="36"/>
+      <c r="C21" s="33"/>
       <c r="D21" s="8">
         <v>0</v>
       </c>
@@ -3740,8 +3738,8 @@
       </c>
     </row>
     <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
       <c r="D22" s="8"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
@@ -3779,8 +3777,8 @@
       </c>
     </row>
     <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="33"/>
-      <c r="C23" s="34"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="8"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
@@ -3818,8 +3816,8 @@
       </c>
     </row>
     <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="8"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
@@ -3857,8 +3855,8 @@
       </c>
     </row>
     <row r="25" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -3892,8 +3890,8 @@
       <c r="AH25" s="3"/>
     </row>
     <row r="26" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -3929,8 +3927,8 @@
       <c r="AH26" s="3"/>
     </row>
     <row r="27" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -3966,8 +3964,8 @@
       <c r="AH27" s="3"/>
     </row>
     <row r="28" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -3985,27 +3983,27 @@
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
-      <c r="U28" s="29" t="s">
+      <c r="U28" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="V28" s="29"/>
-      <c r="W28" s="29"/>
-      <c r="X28" s="29"/>
-      <c r="Y28" s="29"/>
-      <c r="Z28" s="29"/>
-      <c r="AA28" s="29"/>
-      <c r="AB28" s="29"/>
-      <c r="AC28" s="29"/>
-      <c r="AD28" s="29"/>
-      <c r="AE28" s="29"/>
-      <c r="AF28" s="29"/>
-      <c r="AG28" s="29"/>
-      <c r="AH28" s="29"/>
-      <c r="AI28" s="29"/>
+      <c r="V28" s="35"/>
+      <c r="W28" s="35"/>
+      <c r="X28" s="35"/>
+      <c r="Y28" s="35"/>
+      <c r="Z28" s="35"/>
+      <c r="AA28" s="35"/>
+      <c r="AB28" s="35"/>
+      <c r="AC28" s="35"/>
+      <c r="AD28" s="35"/>
+      <c r="AE28" s="35"/>
+      <c r="AF28" s="35"/>
+      <c r="AG28" s="35"/>
+      <c r="AH28" s="35"/>
+      <c r="AI28" s="35"/>
     </row>
     <row r="29" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
@@ -4039,8 +4037,8 @@
       <c r="AH29" s="3"/>
     </row>
     <row r="30" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
@@ -4074,8 +4072,8 @@
       <c r="AH30" s="3"/>
     </row>
     <row r="31" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -4112,8 +4110,8 @@
       </c>
     </row>
     <row r="32" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -4147,8 +4145,8 @@
       <c r="AH32" s="3"/>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -4168,8 +4166,8 @@
       <c r="T33" s="3"/>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -4190,22 +4188,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B21:C21"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="U28:AI28"/>
@@ -4222,6 +4204,22 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -4244,97 +4242,97 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="30"/>
-      <c r="S3" s="30"/>
-      <c r="T3" s="30"/>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="36"/>
+      <c r="V3" s="36"/>
     </row>
     <row r="4" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I4" s="30" t="s">
+      <c r="I4" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="30"/>
-      <c r="T4" s="30"/>
-      <c r="U4" s="30"/>
-      <c r="V4" s="30"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
     </row>
     <row r="5" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I5" s="30" t="s">
+      <c r="I5" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="36"/>
+      <c r="R5" s="36"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="36"/>
+      <c r="U5" s="36"/>
+      <c r="V5" s="36"/>
     </row>
     <row r="6" spans="2:35" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I6" s="31" t="s">
+      <c r="I6" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="31"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="31"/>
-      <c r="S6" s="31"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="31"/>
-      <c r="V6" s="31"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
+      <c r="S6" s="37"/>
+      <c r="T6" s="37"/>
+      <c r="U6" s="37"/>
+      <c r="V6" s="37"/>
     </row>
     <row r="7" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="K7" s="27" t="s">
+      <c r="K7" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="L7" s="27"/>
-      <c r="M7" s="27"/>
-      <c r="N7" s="27"/>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="27"/>
-      <c r="T7" s="27"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="34"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="34"/>
+      <c r="S7" s="34"/>
+      <c r="T7" s="34"/>
     </row>
     <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="37" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="37"/>
+      <c r="B9" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="28"/>
       <c r="D9" s="4">
         <v>1</v>
       </c>
@@ -4433,10 +4431,10 @@
       </c>
     </row>
     <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="8">
         <v>0</v>
       </c>
@@ -4536,10 +4534,10 @@
       </c>
     </row>
     <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="32"/>
+      <c r="C11" s="27"/>
       <c r="D11" s="8">
         <v>0</v>
       </c>
@@ -4639,10 +4637,10 @@
       </c>
     </row>
     <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="32"/>
+      <c r="C12" s="27"/>
       <c r="D12" s="8">
         <v>0</v>
       </c>
@@ -4742,10 +4740,10 @@
       </c>
     </row>
     <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="32"/>
+      <c r="C13" s="27"/>
       <c r="D13" s="8">
         <v>0</v>
       </c>
@@ -4845,10 +4843,10 @@
       </c>
     </row>
     <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="32"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="8">
         <v>0</v>
       </c>
@@ -4948,10 +4946,10 @@
       </c>
     </row>
     <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="32"/>
+      <c r="C15" s="27"/>
       <c r="D15" s="8">
         <v>0</v>
       </c>
@@ -5051,10 +5049,10 @@
       </c>
     </row>
     <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="32"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="8">
         <v>0</v>
       </c>
@@ -5154,10 +5152,10 @@
       </c>
     </row>
     <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="32"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="8">
         <v>0</v>
       </c>
@@ -5257,10 +5255,10 @@
       </c>
     </row>
     <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="C18" s="32"/>
+      <c r="C18" s="27"/>
       <c r="D18" s="8">
         <v>0</v>
       </c>
@@ -5360,10 +5358,10 @@
       </c>
     </row>
     <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="32"/>
+      <c r="C19" s="27"/>
       <c r="D19" s="8">
         <v>0</v>
       </c>
@@ -5463,10 +5461,10 @@
       </c>
     </row>
     <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="32"/>
+      <c r="C20" s="27"/>
       <c r="D20" s="8">
         <v>0</v>
       </c>
@@ -5566,10 +5564,10 @@
       </c>
     </row>
     <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="32"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="8">
         <v>0</v>
       </c>
@@ -5772,10 +5770,10 @@
       </c>
     </row>
     <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="36"/>
+      <c r="C23" s="33"/>
       <c r="D23" s="8">
         <v>0</v>
       </c>
@@ -5875,10 +5873,10 @@
       </c>
     </row>
     <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="35" t="s">
+      <c r="B24" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="36"/>
+      <c r="C24" s="33"/>
       <c r="D24" s="8">
         <v>0</v>
       </c>
@@ -5978,10 +5976,10 @@
       </c>
     </row>
     <row r="25" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="35" t="s">
+      <c r="B25" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="36"/>
+      <c r="C25" s="33"/>
       <c r="D25" s="8">
         <v>0</v>
       </c>
@@ -6081,10 +6079,10 @@
       </c>
     </row>
     <row r="26" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="35" t="s">
+      <c r="B26" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="36"/>
+      <c r="C26" s="33"/>
       <c r="D26" s="8">
         <v>0</v>
       </c>
@@ -6184,10 +6182,10 @@
       </c>
     </row>
     <row r="27" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="36"/>
+      <c r="C27" s="33"/>
       <c r="D27" s="8">
         <v>0</v>
       </c>
@@ -6287,10 +6285,10 @@
       </c>
     </row>
     <row r="28" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="35" t="s">
+      <c r="B28" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="36"/>
+      <c r="C28" s="33"/>
       <c r="D28" s="8">
         <v>0</v>
       </c>
@@ -6390,10 +6388,10 @@
       </c>
     </row>
     <row r="29" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="C29" s="36"/>
+      <c r="C29" s="33"/>
       <c r="D29" s="8">
         <v>0</v>
       </c>
@@ -6493,8 +6491,8 @@
       </c>
     </row>
     <row r="30" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="35"/>
-      <c r="C30" s="36"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="33"/>
       <c r="D30" s="24"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
@@ -6527,12 +6525,13 @@
       <c r="AG30" s="9"/>
       <c r="AH30" s="25"/>
       <c r="AI30" s="11">
-        <v>746</v>
+        <f>SUM(AI10:AI29)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -6568,10 +6567,11 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
+      <c r="AI31" s="84"/>
     </row>
     <row r="32" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -6607,8 +6607,8 @@
       <c r="AH32" s="3"/>
     </row>
     <row r="33" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -6626,27 +6626,27 @@
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
-      <c r="U33" s="29" t="s">
+      <c r="U33" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="V33" s="29"/>
-      <c r="W33" s="29"/>
-      <c r="X33" s="29"/>
-      <c r="Y33" s="29"/>
-      <c r="Z33" s="29"/>
-      <c r="AA33" s="29"/>
-      <c r="AB33" s="29"/>
-      <c r="AC33" s="29"/>
-      <c r="AD33" s="29"/>
-      <c r="AE33" s="29"/>
-      <c r="AF33" s="29"/>
-      <c r="AG33" s="29"/>
-      <c r="AH33" s="29"/>
-      <c r="AI33" s="29"/>
+      <c r="V33" s="35"/>
+      <c r="W33" s="35"/>
+      <c r="X33" s="35"/>
+      <c r="Y33" s="35"/>
+      <c r="Z33" s="35"/>
+      <c r="AA33" s="35"/>
+      <c r="AB33" s="35"/>
+      <c r="AC33" s="35"/>
+      <c r="AD33" s="35"/>
+      <c r="AE33" s="35"/>
+      <c r="AF33" s="35"/>
+      <c r="AG33" s="35"/>
+      <c r="AH33" s="35"/>
+      <c r="AI33" s="35"/>
     </row>
     <row r="34" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -6680,8 +6680,8 @@
       <c r="AH34" s="3"/>
     </row>
     <row r="35" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -6715,8 +6715,8 @@
       <c r="AH35" s="3"/>
     </row>
     <row r="36" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -6753,8 +6753,8 @@
       </c>
     </row>
     <row r="37" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -6788,8 +6788,8 @@
       <c r="AH37" s="3"/>
     </row>
     <row r="38" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -6809,8 +6809,8 @@
       <c r="T38" s="3"/>
     </row>
     <row r="39" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B39" s="28"/>
-      <c r="C39" s="28"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -6830,8 +6830,8 @@
       <c r="T39" s="3"/>
     </row>
     <row r="40" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -6852,12 +6852,26 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="I3:V3"/>
-    <mergeCell ref="I4:V4"/>
-    <mergeCell ref="I5:V5"/>
-    <mergeCell ref="I6:V6"/>
-    <mergeCell ref="K7:T7"/>
+    <mergeCell ref="U33:AI33"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
@@ -6870,26 +6884,12 @@
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="U33:AI33"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="I3:V3"/>
+    <mergeCell ref="I4:V4"/>
+    <mergeCell ref="I5:V5"/>
+    <mergeCell ref="I6:V6"/>
+    <mergeCell ref="K7:T7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -6921,90 +6921,90 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="31"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="34" t="s">
         <v>135</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" s="14" t="s">
@@ -7609,16 +7609,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="I31:M31"/>
+    <mergeCell ref="B10:B17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B19:B26"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="C6:L6"/>
-    <mergeCell ref="I31:M31"/>
-    <mergeCell ref="B10:B17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B19:B26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -7646,12 +7646,12 @@
       <c r="R2" s="18"/>
     </row>
     <row r="3" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
       <c r="H3" s="18"/>
       <c r="I3" s="18"/>
       <c r="K3" s="18"/>
@@ -7664,14 +7664,14 @@
       <c r="R3" s="18"/>
     </row>
     <row r="4" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
       <c r="I4" s="18"/>
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
@@ -7683,14 +7683,14 @@
       <c r="R4" s="18"/>
     </row>
     <row r="5" spans="3:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
       <c r="I5" s="19"/>
       <c r="K5" s="19"/>
       <c r="L5" s="19"/>
@@ -7702,24 +7702,24 @@
       <c r="R5" s="19"/>
     </row>
     <row r="6" spans="3:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
     </row>
     <row r="7" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
       <c r="I7" s="20"/>
       <c r="J7" s="20"/>
       <c r="K7" s="20"/>
@@ -7777,10 +7777,10 @@
       </c>
       <c r="E13" s="51"/>
       <c r="F13" s="51"/>
-      <c r="G13" s="84">
-        <v>0</v>
-      </c>
-      <c r="H13" s="84">
+      <c r="G13" s="12">
+        <v>0</v>
+      </c>
+      <c r="H13" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7790,10 +7790,10 @@
       </c>
       <c r="E14" s="51"/>
       <c r="F14" s="51"/>
-      <c r="G14" s="84">
-        <v>0</v>
-      </c>
-      <c r="H14" s="84">
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7803,10 +7803,10 @@
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="51"/>
-      <c r="G15" s="84">
-        <v>0</v>
-      </c>
-      <c r="H15" s="84">
+      <c r="G15" s="12">
+        <v>0</v>
+      </c>
+      <c r="H15" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7816,10 +7816,10 @@
       </c>
       <c r="E16" s="51"/>
       <c r="F16" s="51"/>
-      <c r="G16" s="84">
-        <v>0</v>
-      </c>
-      <c r="H16" s="84">
+      <c r="G16" s="12">
+        <v>0</v>
+      </c>
+      <c r="H16" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7829,10 +7829,10 @@
       </c>
       <c r="E17" s="53"/>
       <c r="F17" s="54"/>
-      <c r="G17" s="84">
-        <v>0</v>
-      </c>
-      <c r="H17" s="84">
+      <c r="G17" s="12">
+        <v>0</v>
+      </c>
+      <c r="H17" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7842,10 +7842,10 @@
       </c>
       <c r="E18" s="51"/>
       <c r="F18" s="51"/>
-      <c r="G18" s="84">
-        <v>0</v>
-      </c>
-      <c r="H18" s="84">
+      <c r="G18" s="12">
+        <v>0</v>
+      </c>
+      <c r="H18" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7918,37 +7918,37 @@
   </cols>
   <sheetData>
     <row r="3" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
     </row>
     <row r="4" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
     </row>
     <row r="5" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
       <c r="O5" s="18"/>
@@ -7976,15 +7976,15 @@
       <c r="S6" s="18"/>
     </row>
     <row r="7" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="27"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
       <c r="M7" s="18"/>
       <c r="N7" s="18"/>
       <c r="O7" s="18"/>
@@ -8008,159 +8008,159 @@
       <c r="S8" s="19"/>
     </row>
     <row r="10" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F10" s="58" t="s">
+      <c r="F10" s="59" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
-      <c r="K10" s="59"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="60"/>
     </row>
     <row r="11" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="63"/>
-      <c r="J11" s="65" t="s">
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="K11" s="65"/>
+      <c r="K11" s="56"/>
     </row>
     <row r="12" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F12" s="64" t="s">
+      <c r="F12" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="64"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="65">
-        <v>0</v>
-      </c>
-      <c r="K12" s="65"/>
+      <c r="G12" s="57"/>
+      <c r="H12" s="57"/>
+      <c r="I12" s="57"/>
+      <c r="J12" s="56">
+        <v>0</v>
+      </c>
+      <c r="K12" s="56"/>
     </row>
     <row r="13" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F13" s="64" t="s">
+      <c r="F13" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="G13" s="64"/>
-      <c r="H13" s="64"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="65">
-        <v>0</v>
-      </c>
-      <c r="K13" s="65"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="57"/>
+      <c r="I13" s="57"/>
+      <c r="J13" s="56">
+        <v>0</v>
+      </c>
+      <c r="K13" s="56"/>
     </row>
     <row r="14" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F14" s="64" t="s">
+      <c r="F14" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="G14" s="64"/>
-      <c r="H14" s="64"/>
-      <c r="I14" s="64"/>
-      <c r="J14" s="65">
-        <v>0</v>
-      </c>
-      <c r="K14" s="65"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
+      <c r="I14" s="57"/>
+      <c r="J14" s="56">
+        <v>0</v>
+      </c>
+      <c r="K14" s="56"/>
     </row>
     <row r="15" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F15" s="64" t="s">
+      <c r="F15" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
-      <c r="J15" s="65">
-        <v>0</v>
-      </c>
-      <c r="K15" s="65"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="57"/>
+      <c r="J15" s="56">
+        <v>0</v>
+      </c>
+      <c r="K15" s="56"/>
     </row>
     <row r="16" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F16" s="64" t="s">
+      <c r="F16" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="G16" s="64"/>
-      <c r="H16" s="64"/>
-      <c r="I16" s="64"/>
-      <c r="J16" s="65">
-        <v>0</v>
-      </c>
-      <c r="K16" s="65"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="56">
+        <v>0</v>
+      </c>
+      <c r="K16" s="56"/>
     </row>
     <row r="17" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F17" s="55" t="s">
+      <c r="F17" s="61" t="s">
         <v>83</v>
       </c>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="58">
-        <v>0</v>
-      </c>
-      <c r="K17" s="59"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="63"/>
+      <c r="J17" s="59">
+        <v>0</v>
+      </c>
+      <c r="K17" s="60"/>
     </row>
     <row r="18" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F18" s="64" t="s">
+      <c r="F18" s="57" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="64"/>
-      <c r="H18" s="64"/>
-      <c r="I18" s="64"/>
-      <c r="J18" s="65">
-        <v>0</v>
-      </c>
-      <c r="K18" s="65"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="57"/>
+      <c r="J18" s="56">
+        <v>0</v>
+      </c>
+      <c r="K18" s="56"/>
     </row>
     <row r="19" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="58">
-        <v>0</v>
-      </c>
-      <c r="K19" s="59"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="59">
+        <v>0</v>
+      </c>
+      <c r="K19" s="60"/>
     </row>
     <row r="20" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F20" s="55"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="59"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="60"/>
     </row>
     <row r="21" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F21" s="55"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="57"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="59"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="63"/>
+      <c r="J21" s="59"/>
+      <c r="K21" s="60"/>
     </row>
     <row r="22" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="65"/>
-      <c r="K22" s="65"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
     </row>
     <row r="23" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F23" s="65" t="s">
+      <c r="F23" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="G23" s="65"/>
-      <c r="H23" s="65"/>
-      <c r="I23" s="65"/>
-      <c r="J23" s="65">
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56">
         <f>SUM(J12:K22)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="65"/>
+      <c r="K23" s="56"/>
     </row>
     <row r="27" spans="6:15" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
@@ -8176,9 +8176,9 @@
       <c r="J29" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="K29" s="66"/>
-      <c r="L29" s="66"/>
-      <c r="M29" s="66"/>
+      <c r="K29" s="55"/>
+      <c r="L29" s="55"/>
+      <c r="M29" s="55"/>
     </row>
     <row r="31" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O31" t="s">
@@ -8187,6 +8187,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="F7:L7"/>
+    <mergeCell ref="F3:L3"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="F5:L5"/>
+    <mergeCell ref="F10:K10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
     <mergeCell ref="J29:M29"/>
     <mergeCell ref="F23:I23"/>
     <mergeCell ref="J23:K23"/>
@@ -8203,22 +8219,6 @@
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="F17:I17"/>
     <mergeCell ref="F21:I21"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="F7:L7"/>
-    <mergeCell ref="F3:L3"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="F5:L5"/>
-    <mergeCell ref="F10:K10"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8246,85 +8246,85 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C6" s="75" t="s">
+      <c r="C6" s="68" t="s">
         <v>133</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B9" s="14" t="s">
@@ -8333,10 +8333,10 @@
       <c r="C9" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="74" t="s">
+      <c r="D9" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="E9" s="74"/>
+      <c r="E9" s="69"/>
       <c r="F9" s="70" t="s">
         <v>51</v>
       </c>
@@ -8345,10 +8345,10 @@
         <v>52</v>
       </c>
       <c r="I9" s="70"/>
-      <c r="J9" s="71" t="s">
+      <c r="J9" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="K9" s="72"/>
+      <c r="K9" s="73"/>
       <c r="L9" s="14" t="s">
         <v>32</v>
       </c>
@@ -8364,18 +8364,18 @@
         <v>0</v>
       </c>
       <c r="E10" s="70"/>
-      <c r="F10" s="73">
-        <v>0</v>
-      </c>
-      <c r="G10" s="73"/>
+      <c r="F10" s="71">
+        <v>0</v>
+      </c>
+      <c r="G10" s="71"/>
       <c r="H10" s="70">
         <v>0</v>
       </c>
       <c r="I10" s="70"/>
-      <c r="J10" s="68">
-        <v>0</v>
-      </c>
-      <c r="K10" s="69"/>
+      <c r="J10" s="74">
+        <v>0</v>
+      </c>
+      <c r="K10" s="75"/>
       <c r="L10" s="2">
         <f t="shared" ref="L10:L17" si="0">SUM(D10:K10)</f>
         <v>0</v>
@@ -8390,18 +8390,18 @@
         <v>0</v>
       </c>
       <c r="E11" s="70"/>
-      <c r="F11" s="73">
-        <v>0</v>
-      </c>
-      <c r="G11" s="73"/>
+      <c r="F11" s="71">
+        <v>0</v>
+      </c>
+      <c r="G11" s="71"/>
       <c r="H11" s="70">
         <v>0</v>
       </c>
       <c r="I11" s="70"/>
-      <c r="J11" s="68">
-        <v>0</v>
-      </c>
-      <c r="K11" s="69"/>
+      <c r="J11" s="74">
+        <v>0</v>
+      </c>
+      <c r="K11" s="75"/>
       <c r="L11" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8416,18 +8416,18 @@
         <v>0</v>
       </c>
       <c r="E12" s="70"/>
-      <c r="F12" s="73">
-        <v>0</v>
-      </c>
-      <c r="G12" s="73"/>
+      <c r="F12" s="71">
+        <v>0</v>
+      </c>
+      <c r="G12" s="71"/>
       <c r="H12" s="70">
         <v>0</v>
       </c>
       <c r="I12" s="70"/>
-      <c r="J12" s="68">
-        <v>0</v>
-      </c>
-      <c r="K12" s="69"/>
+      <c r="J12" s="74">
+        <v>0</v>
+      </c>
+      <c r="K12" s="75"/>
       <c r="L12" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8442,18 +8442,18 @@
         <v>0</v>
       </c>
       <c r="E13" s="70"/>
-      <c r="F13" s="73">
-        <v>0</v>
-      </c>
-      <c r="G13" s="73"/>
+      <c r="F13" s="71">
+        <v>0</v>
+      </c>
+      <c r="G13" s="71"/>
       <c r="H13" s="70">
         <v>0</v>
       </c>
       <c r="I13" s="70"/>
-      <c r="J13" s="68">
-        <v>0</v>
-      </c>
-      <c r="K13" s="69"/>
+      <c r="J13" s="74">
+        <v>0</v>
+      </c>
+      <c r="K13" s="75"/>
       <c r="L13" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8468,18 +8468,18 @@
         <v>0</v>
       </c>
       <c r="E14" s="70"/>
-      <c r="F14" s="73">
-        <v>0</v>
-      </c>
-      <c r="G14" s="73"/>
+      <c r="F14" s="71">
+        <v>0</v>
+      </c>
+      <c r="G14" s="71"/>
       <c r="H14" s="70">
         <v>0</v>
       </c>
       <c r="I14" s="70"/>
-      <c r="J14" s="68">
-        <v>0</v>
-      </c>
-      <c r="K14" s="69"/>
+      <c r="J14" s="74">
+        <v>0</v>
+      </c>
+      <c r="K14" s="75"/>
       <c r="L14" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8494,18 +8494,18 @@
         <v>0</v>
       </c>
       <c r="E15" s="70"/>
-      <c r="F15" s="73">
-        <v>0</v>
-      </c>
-      <c r="G15" s="73"/>
+      <c r="F15" s="71">
+        <v>0</v>
+      </c>
+      <c r="G15" s="71"/>
       <c r="H15" s="70">
         <v>0</v>
       </c>
       <c r="I15" s="70"/>
-      <c r="J15" s="68">
-        <v>0</v>
-      </c>
-      <c r="K15" s="69"/>
+      <c r="J15" s="74">
+        <v>0</v>
+      </c>
+      <c r="K15" s="75"/>
       <c r="L15" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8520,18 +8520,18 @@
         <v>0</v>
       </c>
       <c r="E16" s="70"/>
-      <c r="F16" s="73">
-        <v>0</v>
-      </c>
-      <c r="G16" s="73"/>
+      <c r="F16" s="71">
+        <v>0</v>
+      </c>
+      <c r="G16" s="71"/>
       <c r="H16" s="70">
         <v>0</v>
       </c>
       <c r="I16" s="70"/>
-      <c r="J16" s="68">
-        <v>0</v>
-      </c>
-      <c r="K16" s="69"/>
+      <c r="J16" s="74">
+        <v>0</v>
+      </c>
+      <c r="K16" s="75"/>
       <c r="L16" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8546,18 +8546,18 @@
         <v>0</v>
       </c>
       <c r="E17" s="70"/>
-      <c r="F17" s="73">
-        <v>0</v>
-      </c>
-      <c r="G17" s="73"/>
+      <c r="F17" s="71">
+        <v>0</v>
+      </c>
+      <c r="G17" s="71"/>
       <c r="H17" s="70">
         <v>0</v>
       </c>
       <c r="I17" s="70"/>
-      <c r="J17" s="68">
-        <v>0</v>
-      </c>
-      <c r="K17" s="69"/>
+      <c r="J17" s="74">
+        <v>0</v>
+      </c>
+      <c r="K17" s="75"/>
       <c r="L17" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -8572,18 +8572,18 @@
         <v>0</v>
       </c>
       <c r="E18" s="70"/>
-      <c r="F18" s="73">
-        <v>0</v>
-      </c>
-      <c r="G18" s="73"/>
+      <c r="F18" s="71">
+        <v>0</v>
+      </c>
+      <c r="G18" s="71"/>
       <c r="H18" s="70">
         <v>0</v>
       </c>
       <c r="I18" s="70"/>
-      <c r="J18" s="68">
-        <v>0</v>
-      </c>
-      <c r="K18" s="69"/>
+      <c r="J18" s="74">
+        <v>0</v>
+      </c>
+      <c r="K18" s="75"/>
       <c r="L18" s="2">
         <f>SUM(L10:L17)</f>
         <v>0</v>
@@ -8600,18 +8600,18 @@
         <v>0</v>
       </c>
       <c r="E19" s="70"/>
-      <c r="F19" s="73">
-        <v>0</v>
-      </c>
-      <c r="G19" s="73"/>
+      <c r="F19" s="71">
+        <v>0</v>
+      </c>
+      <c r="G19" s="71"/>
       <c r="H19" s="70">
         <v>0</v>
       </c>
       <c r="I19" s="70"/>
-      <c r="J19" s="68">
-        <v>0</v>
-      </c>
-      <c r="K19" s="69"/>
+      <c r="J19" s="74">
+        <v>0</v>
+      </c>
+      <c r="K19" s="75"/>
       <c r="L19" s="2">
         <f t="shared" ref="L19:L26" si="1">SUM(D19:K19)</f>
         <v>0</v>
@@ -8626,18 +8626,18 @@
         <v>0</v>
       </c>
       <c r="E20" s="70"/>
-      <c r="F20" s="73">
-        <v>0</v>
-      </c>
-      <c r="G20" s="73"/>
+      <c r="F20" s="71">
+        <v>0</v>
+      </c>
+      <c r="G20" s="71"/>
       <c r="H20" s="70">
         <v>0</v>
       </c>
       <c r="I20" s="70"/>
-      <c r="J20" s="68">
-        <v>0</v>
-      </c>
-      <c r="K20" s="69"/>
+      <c r="J20" s="74">
+        <v>0</v>
+      </c>
+      <c r="K20" s="75"/>
       <c r="L20" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8652,18 +8652,18 @@
         <v>0</v>
       </c>
       <c r="E21" s="70"/>
-      <c r="F21" s="73">
-        <v>0</v>
-      </c>
-      <c r="G21" s="73"/>
+      <c r="F21" s="71">
+        <v>0</v>
+      </c>
+      <c r="G21" s="71"/>
       <c r="H21" s="70">
         <v>0</v>
       </c>
       <c r="I21" s="70"/>
-      <c r="J21" s="68">
-        <v>0</v>
-      </c>
-      <c r="K21" s="69"/>
+      <c r="J21" s="74">
+        <v>0</v>
+      </c>
+      <c r="K21" s="75"/>
       <c r="L21" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8678,18 +8678,18 @@
         <v>0</v>
       </c>
       <c r="E22" s="70"/>
-      <c r="F22" s="73">
-        <v>0</v>
-      </c>
-      <c r="G22" s="73"/>
+      <c r="F22" s="71">
+        <v>0</v>
+      </c>
+      <c r="G22" s="71"/>
       <c r="H22" s="70">
         <v>0</v>
       </c>
       <c r="I22" s="70"/>
-      <c r="J22" s="68">
-        <v>0</v>
-      </c>
-      <c r="K22" s="69"/>
+      <c r="J22" s="74">
+        <v>0</v>
+      </c>
+      <c r="K22" s="75"/>
       <c r="L22" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8704,18 +8704,18 @@
         <v>0</v>
       </c>
       <c r="E23" s="70"/>
-      <c r="F23" s="73">
-        <v>0</v>
-      </c>
-      <c r="G23" s="73"/>
+      <c r="F23" s="71">
+        <v>0</v>
+      </c>
+      <c r="G23" s="71"/>
       <c r="H23" s="70">
         <v>0</v>
       </c>
       <c r="I23" s="70"/>
-      <c r="J23" s="68">
-        <v>0</v>
-      </c>
-      <c r="K23" s="69"/>
+      <c r="J23" s="74">
+        <v>0</v>
+      </c>
+      <c r="K23" s="75"/>
       <c r="L23" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8730,18 +8730,18 @@
         <v>0</v>
       </c>
       <c r="E24" s="70"/>
-      <c r="F24" s="73">
-        <v>0</v>
-      </c>
-      <c r="G24" s="73"/>
+      <c r="F24" s="71">
+        <v>0</v>
+      </c>
+      <c r="G24" s="71"/>
       <c r="H24" s="70">
         <v>0</v>
       </c>
       <c r="I24" s="70"/>
-      <c r="J24" s="68">
-        <v>0</v>
-      </c>
-      <c r="K24" s="69"/>
+      <c r="J24" s="74">
+        <v>0</v>
+      </c>
+      <c r="K24" s="75"/>
       <c r="L24" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8756,18 +8756,18 @@
         <v>0</v>
       </c>
       <c r="E25" s="70"/>
-      <c r="F25" s="73">
-        <v>0</v>
-      </c>
-      <c r="G25" s="73"/>
+      <c r="F25" s="71">
+        <v>0</v>
+      </c>
+      <c r="G25" s="71"/>
       <c r="H25" s="70">
         <v>0</v>
       </c>
       <c r="I25" s="70"/>
-      <c r="J25" s="68">
-        <v>0</v>
-      </c>
-      <c r="K25" s="69"/>
+      <c r="J25" s="74">
+        <v>0</v>
+      </c>
+      <c r="K25" s="75"/>
       <c r="L25" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8782,18 +8782,18 @@
         <v>0</v>
       </c>
       <c r="E26" s="70"/>
-      <c r="F26" s="73">
-        <v>0</v>
-      </c>
-      <c r="G26" s="73"/>
+      <c r="F26" s="71">
+        <v>0</v>
+      </c>
+      <c r="G26" s="71"/>
       <c r="H26" s="70">
         <v>0</v>
       </c>
       <c r="I26" s="70"/>
-      <c r="J26" s="68">
-        <v>0</v>
-      </c>
-      <c r="K26" s="69"/>
+      <c r="J26" s="74">
+        <v>0</v>
+      </c>
+      <c r="K26" s="75"/>
       <c r="L26" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -8808,18 +8808,18 @@
         <v>0</v>
       </c>
       <c r="E27" s="70"/>
-      <c r="F27" s="73">
-        <v>0</v>
-      </c>
-      <c r="G27" s="73"/>
+      <c r="F27" s="71">
+        <v>0</v>
+      </c>
+      <c r="G27" s="71"/>
       <c r="H27" s="70">
         <v>0</v>
       </c>
       <c r="I27" s="70"/>
-      <c r="J27" s="68">
-        <v>0</v>
-      </c>
-      <c r="K27" s="69"/>
+      <c r="J27" s="74">
+        <v>0</v>
+      </c>
+      <c r="K27" s="75"/>
       <c r="L27" s="2">
         <f>SUM(L19:L26)</f>
         <v>0</v>
@@ -8850,11 +8850,71 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:B26"/>
     <mergeCell ref="B27:C27"/>
@@ -8871,71 +8931,11 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C6:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8955,13 +8955,13 @@
   </cols>
   <sheetData>
     <row r="3" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
       <c r="J3" s="18"/>
       <c r="K3" s="18"/>
       <c r="L3" s="18"/>
@@ -8974,14 +8974,14 @@
       <c r="S3" s="18"/>
     </row>
     <row r="4" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
@@ -8993,14 +8993,14 @@
       <c r="S4" s="18"/>
     </row>
     <row r="5" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -9012,14 +9012,14 @@
       <c r="S5" s="18"/>
     </row>
     <row r="6" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
       <c r="K6" s="19"/>
       <c r="L6" s="19"/>
       <c r="M6" s="19"/>
@@ -9031,14 +9031,14 @@
       <c r="S6" s="19"/>
     </row>
     <row r="7" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
     </row>
     <row r="9" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E9" s="70" t="s">
@@ -9057,10 +9057,10 @@
       <c r="F10" s="76"/>
       <c r="G10" s="76"/>
       <c r="H10" s="76"/>
-      <c r="I10" s="65">
-        <v>0</v>
-      </c>
-      <c r="J10" s="65"/>
+      <c r="I10" s="56">
+        <v>0</v>
+      </c>
+      <c r="J10" s="56"/>
     </row>
     <row r="11" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E11" s="76" t="s">
@@ -9069,10 +9069,10 @@
       <c r="F11" s="76"/>
       <c r="G11" s="76"/>
       <c r="H11" s="76"/>
-      <c r="I11" s="65">
-        <v>0</v>
-      </c>
-      <c r="J11" s="65"/>
+      <c r="I11" s="56">
+        <v>0</v>
+      </c>
+      <c r="J11" s="56"/>
     </row>
     <row r="12" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E12" s="76" t="s">
@@ -9081,10 +9081,10 @@
       <c r="F12" s="76"/>
       <c r="G12" s="76"/>
       <c r="H12" s="76"/>
-      <c r="I12" s="65">
-        <v>0</v>
-      </c>
-      <c r="J12" s="65"/>
+      <c r="I12" s="56">
+        <v>0</v>
+      </c>
+      <c r="J12" s="56"/>
     </row>
     <row r="13" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E13" s="76" t="s">
@@ -9093,10 +9093,10 @@
       <c r="F13" s="76"/>
       <c r="G13" s="76"/>
       <c r="H13" s="76"/>
-      <c r="I13" s="65">
-        <v>0</v>
-      </c>
-      <c r="J13" s="65"/>
+      <c r="I13" s="56">
+        <v>0</v>
+      </c>
+      <c r="J13" s="56"/>
     </row>
     <row r="14" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E14" s="76" t="s">
@@ -9105,10 +9105,10 @@
       <c r="F14" s="76"/>
       <c r="G14" s="76"/>
       <c r="H14" s="76"/>
-      <c r="I14" s="65">
-        <v>0</v>
-      </c>
-      <c r="J14" s="65"/>
+      <c r="I14" s="56">
+        <v>0</v>
+      </c>
+      <c r="J14" s="56"/>
     </row>
     <row r="15" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E15" s="76" t="s">
@@ -9117,10 +9117,10 @@
       <c r="F15" s="76"/>
       <c r="G15" s="76"/>
       <c r="H15" s="76"/>
-      <c r="I15" s="65">
-        <v>0</v>
-      </c>
-      <c r="J15" s="65"/>
+      <c r="I15" s="56">
+        <v>0</v>
+      </c>
+      <c r="J15" s="56"/>
     </row>
     <row r="16" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E16" s="77" t="s">
@@ -9129,10 +9129,10 @@
       <c r="F16" s="77"/>
       <c r="G16" s="77"/>
       <c r="H16" s="77"/>
-      <c r="I16" s="65">
-        <v>0</v>
-      </c>
-      <c r="J16" s="65"/>
+      <c r="I16" s="56">
+        <v>0</v>
+      </c>
+      <c r="J16" s="56"/>
     </row>
     <row r="17" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E17" s="76" t="s">
@@ -9141,10 +9141,10 @@
       <c r="F17" s="76"/>
       <c r="G17" s="76"/>
       <c r="H17" s="76"/>
-      <c r="I17" s="65">
-        <v>0</v>
-      </c>
-      <c r="J17" s="65"/>
+      <c r="I17" s="56">
+        <v>0</v>
+      </c>
+      <c r="J17" s="56"/>
     </row>
     <row r="18" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E18" s="76" t="s">
@@ -9153,10 +9153,10 @@
       <c r="F18" s="76"/>
       <c r="G18" s="76"/>
       <c r="H18" s="76"/>
-      <c r="I18" s="65">
-        <v>0</v>
-      </c>
-      <c r="J18" s="65"/>
+      <c r="I18" s="56">
+        <v>0</v>
+      </c>
+      <c r="J18" s="56"/>
     </row>
     <row r="19" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E19" s="78" t="s">
@@ -9165,10 +9165,10 @@
       <c r="F19" s="79"/>
       <c r="G19" s="79"/>
       <c r="H19" s="80"/>
-      <c r="I19" s="58">
-        <v>0</v>
-      </c>
-      <c r="J19" s="59"/>
+      <c r="I19" s="59">
+        <v>0</v>
+      </c>
+      <c r="J19" s="60"/>
     </row>
     <row r="20" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E20" s="76" t="s">
@@ -9177,10 +9177,10 @@
       <c r="F20" s="76"/>
       <c r="G20" s="76"/>
       <c r="H20" s="76"/>
-      <c r="I20" s="65">
-        <v>0</v>
-      </c>
-      <c r="J20" s="65"/>
+      <c r="I20" s="56">
+        <v>0</v>
+      </c>
+      <c r="J20" s="56"/>
     </row>
     <row r="21" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E21" s="81" t="s">
@@ -9189,10 +9189,10 @@
       <c r="F21" s="82"/>
       <c r="G21" s="82"/>
       <c r="H21" s="83"/>
-      <c r="I21" s="58">
-        <v>0</v>
-      </c>
-      <c r="J21" s="59"/>
+      <c r="I21" s="59">
+        <v>0</v>
+      </c>
+      <c r="J21" s="60"/>
     </row>
     <row r="22" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E22" s="78" t="s">
@@ -9201,11 +9201,11 @@
       <c r="F22" s="79"/>
       <c r="G22" s="79"/>
       <c r="H22" s="80"/>
-      <c r="I22" s="58">
+      <c r="I22" s="59">
         <f>SUM(I20:J21)</f>
         <v>0</v>
       </c>
-      <c r="J22" s="59"/>
+      <c r="J22" s="60"/>
     </row>
     <row r="23" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E23" s="76" t="s">
@@ -9214,10 +9214,10 @@
       <c r="F23" s="76"/>
       <c r="G23" s="76"/>
       <c r="H23" s="76"/>
-      <c r="I23" s="65">
-        <v>0</v>
-      </c>
-      <c r="J23" s="65"/>
+      <c r="I23" s="56">
+        <v>0</v>
+      </c>
+      <c r="J23" s="56"/>
     </row>
     <row r="24" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E24" s="76" t="s">
@@ -9226,10 +9226,10 @@
       <c r="F24" s="76"/>
       <c r="G24" s="76"/>
       <c r="H24" s="76"/>
-      <c r="I24" s="65">
-        <v>0</v>
-      </c>
-      <c r="J24" s="65"/>
+      <c r="I24" s="56">
+        <v>0</v>
+      </c>
+      <c r="J24" s="56"/>
     </row>
     <row r="25" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E25" s="77" t="s">
@@ -9238,11 +9238,11 @@
       <c r="F25" s="77"/>
       <c r="G25" s="77"/>
       <c r="H25" s="77"/>
-      <c r="I25" s="65">
+      <c r="I25" s="56">
         <f>SUM(I23:J24)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="65"/>
+      <c r="J25" s="56"/>
     </row>
     <row r="28" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="H28" t="s">
@@ -9270,6 +9270,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E20:H20"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="E15:H15"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="E17:H17"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I19:J19"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="E3:I3"/>
@@ -9286,28 +9308,6 @@
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E20:H20"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="E15:H15"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="E17:H17"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="E23:H23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I15:J15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: Add external consultation report functionality and enhance Excel report generation with error handling
</commit_message>
<xml_diff>
--- a/backend/api-consulmdregister/storage/app/templates/informe_medico_template.xlsx
+++ b/backend/api-consulmdregister/storage/app/templates/informe_medico_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\CR_Clinik_Reynosa\backend\api-consulmdregister\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38BD2F5-33FF-45D7-8564-1BC06F01079D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAF92BB-33C8-42A1-B3F2-0B93FA2BC3C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2115" yWindow="2115" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SERVICIOS MEDICOS" sheetId="1" r:id="rId1"/>
@@ -1024,7 +1024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1090,14 +1090,24 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1111,16 +1121,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1174,24 +1175,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1200,6 +1183,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1213,16 +1202,25 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1231,10 +1229,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1261,7 +1262,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2313,97 +2314,97 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="31"/>
+      <c r="V3" s="31"/>
     </row>
     <row r="4" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="31"/>
+      <c r="T4" s="31"/>
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
     </row>
     <row r="5" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="36"/>
-      <c r="R5" s="36"/>
-      <c r="S5" s="36"/>
-      <c r="T5" s="36"/>
-      <c r="U5" s="36"/>
-      <c r="V5" s="36"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
     </row>
     <row r="6" spans="2:35" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="37"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="37"/>
-      <c r="P6" s="37"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="37"/>
-      <c r="S6" s="37"/>
-      <c r="T6" s="37"/>
-      <c r="U6" s="37"/>
-      <c r="V6" s="37"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
+      <c r="S6" s="32"/>
+      <c r="T6" s="32"/>
+      <c r="U6" s="32"/>
+      <c r="V6" s="32"/>
     </row>
     <row r="7" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="K7" s="34" t="s">
+      <c r="K7" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="L7" s="34"/>
-      <c r="M7" s="34"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="34"/>
-      <c r="P7" s="34"/>
-      <c r="Q7" s="34"/>
-      <c r="R7" s="34"/>
-      <c r="S7" s="34"/>
-      <c r="T7" s="34"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
     </row>
     <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="28"/>
+      <c r="B9" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="38"/>
       <c r="D9" s="4">
         <v>1</v>
       </c>
@@ -2502,10 +2503,10 @@
       </c>
     </row>
     <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="27"/>
+      <c r="C10" s="33"/>
       <c r="D10" s="8">
         <v>0</v>
       </c>
@@ -2605,10 +2606,10 @@
       </c>
     </row>
     <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="33"/>
       <c r="D11" s="8">
         <v>0</v>
       </c>
@@ -2708,10 +2709,10 @@
       </c>
     </row>
     <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="27"/>
+      <c r="C12" s="33"/>
       <c r="D12" s="8">
         <v>0</v>
       </c>
@@ -2811,10 +2812,10 @@
       </c>
     </row>
     <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="C13" s="27"/>
+      <c r="C13" s="33"/>
       <c r="D13" s="8">
         <v>0</v>
       </c>
@@ -2914,10 +2915,10 @@
       </c>
     </row>
     <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="27"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="8">
         <v>0</v>
       </c>
@@ -3017,10 +3018,10 @@
       </c>
     </row>
     <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="27"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="8">
         <v>0</v>
       </c>
@@ -3120,10 +3121,10 @@
       </c>
     </row>
     <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="27"/>
+      <c r="C16" s="33"/>
       <c r="D16" s="8">
         <v>0</v>
       </c>
@@ -3223,10 +3224,10 @@
       </c>
     </row>
     <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="27"/>
+      <c r="C17" s="33"/>
       <c r="D17" s="8">
         <v>0</v>
       </c>
@@ -3326,10 +3327,10 @@
       </c>
     </row>
     <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="27"/>
+      <c r="C18" s="33"/>
       <c r="D18" s="8">
         <v>0</v>
       </c>
@@ -3429,10 +3430,10 @@
       </c>
     </row>
     <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="27"/>
+      <c r="C19" s="33"/>
       <c r="D19" s="8">
         <v>0</v>
       </c>
@@ -3532,10 +3533,10 @@
       </c>
     </row>
     <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="27"/>
+      <c r="C20" s="33"/>
       <c r="D20" s="8">
         <v>0</v>
       </c>
@@ -3635,10 +3636,10 @@
       </c>
     </row>
     <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="33"/>
+      <c r="C21" s="37"/>
       <c r="D21" s="8">
         <v>0</v>
       </c>
@@ -3738,8 +3739,8 @@
       </c>
     </row>
     <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="35"/>
       <c r="D22" s="8"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
@@ -3777,8 +3778,8 @@
       </c>
     </row>
     <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="35"/>
       <c r="D23" s="8"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
@@ -3816,8 +3817,8 @@
       </c>
     </row>
     <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
       <c r="D24" s="8"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
@@ -3983,23 +3984,23 @@
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
-      <c r="U28" s="35" t="s">
+      <c r="U28" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="V28" s="35"/>
-      <c r="W28" s="35"/>
-      <c r="X28" s="35"/>
-      <c r="Y28" s="35"/>
-      <c r="Z28" s="35"/>
-      <c r="AA28" s="35"/>
-      <c r="AB28" s="35"/>
-      <c r="AC28" s="35"/>
-      <c r="AD28" s="35"/>
-      <c r="AE28" s="35"/>
-      <c r="AF28" s="35"/>
-      <c r="AG28" s="35"/>
-      <c r="AH28" s="35"/>
-      <c r="AI28" s="35"/>
+      <c r="V28" s="30"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="30"/>
+      <c r="Y28" s="30"/>
+      <c r="Z28" s="30"/>
+      <c r="AA28" s="30"/>
+      <c r="AB28" s="30"/>
+      <c r="AC28" s="30"/>
+      <c r="AD28" s="30"/>
+      <c r="AE28" s="30"/>
+      <c r="AF28" s="30"/>
+      <c r="AG28" s="30"/>
+      <c r="AH28" s="30"/>
+      <c r="AI28" s="30"/>
     </row>
     <row r="29" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B29" s="29"/>
@@ -4188,6 +4189,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="U28:AI28"/>
@@ -4204,22 +4221,6 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -4242,97 +4243,97 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="31"/>
+      <c r="V3" s="31"/>
     </row>
     <row r="4" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="31"/>
+      <c r="T4" s="31"/>
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
     </row>
     <row r="5" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="36"/>
-      <c r="R5" s="36"/>
-      <c r="S5" s="36"/>
-      <c r="T5" s="36"/>
-      <c r="U5" s="36"/>
-      <c r="V5" s="36"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
     </row>
     <row r="6" spans="2:35" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="37"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="37"/>
-      <c r="P6" s="37"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="37"/>
-      <c r="S6" s="37"/>
-      <c r="T6" s="37"/>
-      <c r="U6" s="37"/>
-      <c r="V6" s="37"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
+      <c r="S6" s="32"/>
+      <c r="T6" s="32"/>
+      <c r="U6" s="32"/>
+      <c r="V6" s="32"/>
     </row>
     <row r="7" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="K7" s="34" t="s">
+      <c r="K7" s="28" t="s">
         <v>130</v>
       </c>
-      <c r="L7" s="34"/>
-      <c r="M7" s="34"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="34"/>
-      <c r="P7" s="34"/>
-      <c r="Q7" s="34"/>
-      <c r="R7" s="34"/>
-      <c r="S7" s="34"/>
-      <c r="T7" s="34"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
     </row>
     <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="28"/>
+      <c r="B9" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="38"/>
       <c r="D9" s="4">
         <v>1</v>
       </c>
@@ -4431,10 +4432,10 @@
       </c>
     </row>
     <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="27"/>
+      <c r="C10" s="33"/>
       <c r="D10" s="8">
         <v>0</v>
       </c>
@@ -4534,10 +4535,10 @@
       </c>
     </row>
     <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="33"/>
       <c r="D11" s="8">
         <v>0</v>
       </c>
@@ -4637,10 +4638,10 @@
       </c>
     </row>
     <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="27"/>
+      <c r="C12" s="33"/>
       <c r="D12" s="8">
         <v>0</v>
       </c>
@@ -4740,10 +4741,10 @@
       </c>
     </row>
     <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="27"/>
+      <c r="C13" s="33"/>
       <c r="D13" s="8">
         <v>0</v>
       </c>
@@ -4843,10 +4844,10 @@
       </c>
     </row>
     <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="27"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="8">
         <v>0</v>
       </c>
@@ -4946,10 +4947,10 @@
       </c>
     </row>
     <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="27"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="8">
         <v>0</v>
       </c>
@@ -5049,10 +5050,10 @@
       </c>
     </row>
     <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="33" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="27"/>
+      <c r="C16" s="33"/>
       <c r="D16" s="8">
         <v>0</v>
       </c>
@@ -5152,10 +5153,10 @@
       </c>
     </row>
     <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="27"/>
+      <c r="C17" s="33"/>
       <c r="D17" s="8">
         <v>0</v>
       </c>
@@ -5255,10 +5256,10 @@
       </c>
     </row>
     <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="C18" s="27"/>
+      <c r="C18" s="33"/>
       <c r="D18" s="8">
         <v>0</v>
       </c>
@@ -5358,10 +5359,10 @@
       </c>
     </row>
     <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="27"/>
+      <c r="C19" s="33"/>
       <c r="D19" s="8">
         <v>0</v>
       </c>
@@ -5461,10 +5462,10 @@
       </c>
     </row>
     <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="27"/>
+      <c r="C20" s="33"/>
       <c r="D20" s="8">
         <v>0</v>
       </c>
@@ -5564,10 +5565,10 @@
       </c>
     </row>
     <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="27"/>
+      <c r="C21" s="33"/>
       <c r="D21" s="8">
         <v>0</v>
       </c>
@@ -5667,10 +5668,10 @@
       </c>
     </row>
     <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="39"/>
+      <c r="C22" s="40"/>
       <c r="D22" s="8">
         <v>0</v>
       </c>
@@ -5770,10 +5771,10 @@
       </c>
     </row>
     <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="33"/>
+      <c r="C23" s="37"/>
       <c r="D23" s="8">
         <v>0</v>
       </c>
@@ -5873,10 +5874,10 @@
       </c>
     </row>
     <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="33"/>
+      <c r="C24" s="37"/>
       <c r="D24" s="8">
         <v>0</v>
       </c>
@@ -5976,10 +5977,10 @@
       </c>
     </row>
     <row r="25" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="33"/>
+      <c r="C25" s="37"/>
       <c r="D25" s="8">
         <v>0</v>
       </c>
@@ -6079,10 +6080,10 @@
       </c>
     </row>
     <row r="26" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="33"/>
+      <c r="C26" s="37"/>
       <c r="D26" s="8">
         <v>0</v>
       </c>
@@ -6182,10 +6183,10 @@
       </c>
     </row>
     <row r="27" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="33"/>
+      <c r="C27" s="37"/>
       <c r="D27" s="8">
         <v>0</v>
       </c>
@@ -6285,10 +6286,10 @@
       </c>
     </row>
     <row r="28" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="33"/>
+      <c r="C28" s="37"/>
       <c r="D28" s="8">
         <v>0</v>
       </c>
@@ -6388,10 +6389,10 @@
       </c>
     </row>
     <row r="29" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="36" t="s">
         <v>124</v>
       </c>
-      <c r="C29" s="33"/>
+      <c r="C29" s="37"/>
       <c r="D29" s="8">
         <v>0</v>
       </c>
@@ -6491,8 +6492,8 @@
       </c>
     </row>
     <row r="30" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="32"/>
-      <c r="C30" s="33"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="37"/>
       <c r="D30" s="24"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
@@ -6567,7 +6568,7 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
-      <c r="AI31" s="84"/>
+      <c r="AI31" s="27"/>
     </row>
     <row r="32" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B32" s="29"/>
@@ -6626,23 +6627,23 @@
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
-      <c r="U33" s="35" t="s">
+      <c r="U33" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="V33" s="35"/>
-      <c r="W33" s="35"/>
-      <c r="X33" s="35"/>
-      <c r="Y33" s="35"/>
-      <c r="Z33" s="35"/>
-      <c r="AA33" s="35"/>
-      <c r="AB33" s="35"/>
-      <c r="AC33" s="35"/>
-      <c r="AD33" s="35"/>
-      <c r="AE33" s="35"/>
-      <c r="AF33" s="35"/>
-      <c r="AG33" s="35"/>
-      <c r="AH33" s="35"/>
-      <c r="AI33" s="35"/>
+      <c r="V33" s="30"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="30"/>
+      <c r="Y33" s="30"/>
+      <c r="Z33" s="30"/>
+      <c r="AA33" s="30"/>
+      <c r="AB33" s="30"/>
+      <c r="AC33" s="30"/>
+      <c r="AD33" s="30"/>
+      <c r="AE33" s="30"/>
+      <c r="AF33" s="30"/>
+      <c r="AG33" s="30"/>
+      <c r="AH33" s="30"/>
+      <c r="AI33" s="30"/>
     </row>
     <row r="34" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B34" s="29"/>
@@ -6852,26 +6853,12 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="U33:AI33"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="I3:V3"/>
+    <mergeCell ref="I4:V4"/>
+    <mergeCell ref="I5:V5"/>
+    <mergeCell ref="I6:V6"/>
+    <mergeCell ref="K7:T7"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
@@ -6884,12 +6871,26 @@
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="I3:V3"/>
-    <mergeCell ref="I4:V4"/>
-    <mergeCell ref="I5:V5"/>
-    <mergeCell ref="I6:V6"/>
-    <mergeCell ref="K7:T7"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="U33:AI33"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -6921,90 +6922,90 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" s="14" t="s">
@@ -7057,7 +7058,7 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="42" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="13" t="s">
@@ -7084,7 +7085,7 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="42"/>
+      <c r="B11" s="43"/>
       <c r="C11" s="13" t="s">
         <v>37</v>
       </c>
@@ -7109,7 +7110,7 @@
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="42"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="13" t="s">
         <v>36</v>
       </c>
@@ -7134,7 +7135,7 @@
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="42"/>
+      <c r="B13" s="43"/>
       <c r="C13" s="13" t="s">
         <v>38</v>
       </c>
@@ -7159,7 +7160,7 @@
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="42"/>
+      <c r="B14" s="43"/>
       <c r="C14" s="13" t="s">
         <v>39</v>
       </c>
@@ -7184,7 +7185,7 @@
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="42"/>
+      <c r="B15" s="43"/>
       <c r="C15" s="13" t="s">
         <v>40</v>
       </c>
@@ -7209,7 +7210,7 @@
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="42"/>
+      <c r="B16" s="43"/>
       <c r="C16" s="13" t="s">
         <v>41</v>
       </c>
@@ -7234,7 +7235,7 @@
       </c>
     </row>
     <row r="17" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="42"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="17" t="s">
         <v>42</v>
       </c>
@@ -7259,10 +7260,10 @@
       </c>
     </row>
     <row r="18" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="44"/>
+      <c r="C18" s="45"/>
       <c r="D18" s="2">
         <f t="shared" ref="D18:Q18" si="1">SUM(D10:D17)</f>
         <v>0</v>
@@ -7321,7 +7322,7 @@
       </c>
     </row>
     <row r="19" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="48" t="s">
         <v>34</v>
       </c>
       <c r="C19" s="16" t="s">
@@ -7348,7 +7349,7 @@
       </c>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="48"/>
+      <c r="B20" s="49"/>
       <c r="C20" s="2" t="s">
         <v>37</v>
       </c>
@@ -7373,7 +7374,7 @@
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" s="48"/>
+      <c r="B21" s="49"/>
       <c r="C21" s="2" t="s">
         <v>36</v>
       </c>
@@ -7398,7 +7399,7 @@
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="48"/>
+      <c r="B22" s="49"/>
       <c r="C22" s="2" t="s">
         <v>38</v>
       </c>
@@ -7423,7 +7424,7 @@
       </c>
     </row>
     <row r="23" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B23" s="48"/>
+      <c r="B23" s="49"/>
       <c r="C23" s="2" t="s">
         <v>39</v>
       </c>
@@ -7448,7 +7449,7 @@
       </c>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="48"/>
+      <c r="B24" s="49"/>
       <c r="C24" s="2" t="s">
         <v>40</v>
       </c>
@@ -7473,7 +7474,7 @@
       </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B25" s="48"/>
+      <c r="B25" s="49"/>
       <c r="C25" s="2" t="s">
         <v>41</v>
       </c>
@@ -7498,7 +7499,7 @@
       </c>
     </row>
     <row r="26" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="49"/>
+      <c r="B26" s="50"/>
       <c r="C26" s="15" t="s">
         <v>42</v>
       </c>
@@ -7523,12 +7524,13 @@
       </c>
     </row>
     <row r="27" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="46"/>
+      <c r="C27" s="47"/>
       <c r="D27" s="2">
-        <v>637</v>
+        <f>SUM(D19:D26)</f>
+        <v>0</v>
       </c>
       <c r="E27" s="2">
         <f t="shared" ref="E27:Q27" si="3">SUM(E19:E26)</f>
@@ -7582,6 +7584,9 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+    </row>
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D28" s="85"/>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
@@ -7594,13 +7599,13 @@
       </c>
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="I31" s="40" t="s">
+      <c r="I31" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="40"/>
-      <c r="M31" s="40"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
+      <c r="M31" s="41"/>
     </row>
     <row r="33" spans="16:16" x14ac:dyDescent="0.25">
       <c r="P33" t="s">
@@ -7609,16 +7614,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A5:N5"/>
+    <mergeCell ref="C6:L6"/>
     <mergeCell ref="I31:M31"/>
     <mergeCell ref="B10:B17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B19:B26"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A5:N5"/>
-    <mergeCell ref="C6:L6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -7646,12 +7651,12 @@
       <c r="R2" s="18"/>
     </row>
     <row r="3" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
       <c r="H3" s="18"/>
       <c r="I3" s="18"/>
       <c r="K3" s="18"/>
@@ -7664,14 +7669,14 @@
       <c r="R3" s="18"/>
     </row>
     <row r="4" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
       <c r="I4" s="18"/>
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
@@ -7683,14 +7688,14 @@
       <c r="R4" s="18"/>
     </row>
     <row r="5" spans="3:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
       <c r="I5" s="19"/>
       <c r="K5" s="19"/>
       <c r="L5" s="19"/>
@@ -7702,24 +7707,24 @@
       <c r="R5" s="19"/>
     </row>
     <row r="6" spans="3:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
       <c r="I7" s="20"/>
       <c r="J7" s="20"/>
       <c r="K7" s="20"/>
@@ -7772,11 +7777,11 @@
       </c>
     </row>
     <row r="13" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D13" s="51" t="s">
+      <c r="D13" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="51"/>
-      <c r="F13" s="51"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
       <c r="G13" s="12">
         <v>0</v>
       </c>
@@ -7785,11 +7790,11 @@
       </c>
     </row>
     <row r="14" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D14" s="51" t="s">
+      <c r="D14" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
       <c r="G14" s="12">
         <v>0</v>
       </c>
@@ -7798,11 +7803,11 @@
       </c>
     </row>
     <row r="15" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="51" t="s">
+      <c r="D15" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
       <c r="G15" s="12">
         <v>0</v>
       </c>
@@ -7811,11 +7816,11 @@
       </c>
     </row>
     <row r="16" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="51" t="s">
+      <c r="D16" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="51"/>
-      <c r="F16" s="51"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="52"/>
       <c r="G16" s="12">
         <v>0</v>
       </c>
@@ -7824,11 +7829,11 @@
       </c>
     </row>
     <row r="17" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="52" t="s">
+      <c r="D17" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="53"/>
-      <c r="F17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="55"/>
       <c r="G17" s="12">
         <v>0</v>
       </c>
@@ -7837,11 +7842,11 @@
       </c>
     </row>
     <row r="18" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="51" t="s">
+      <c r="D18" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="51"/>
-      <c r="F18" s="51"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="52"/>
       <c r="G18" s="12">
         <v>0</v>
       </c>
@@ -7873,12 +7878,12 @@
       </c>
     </row>
     <row r="25" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="G25" s="50" t="s">
+      <c r="G25" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="50"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="51"/>
     </row>
     <row r="28" spans="4:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
@@ -7918,37 +7923,37 @@
   </cols>
   <sheetData>
     <row r="3" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F3" s="36" t="s">
+      <c r="F3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
     </row>
     <row r="4" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
     </row>
     <row r="5" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F5" s="36" t="s">
+      <c r="F5" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
       <c r="O5" s="18"/>
@@ -7976,15 +7981,15 @@
       <c r="S6" s="18"/>
     </row>
     <row r="7" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F7" s="34" t="s">
+      <c r="F7" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
       <c r="M7" s="18"/>
       <c r="N7" s="18"/>
       <c r="O7" s="18"/>
@@ -8011,156 +8016,156 @@
       <c r="F10" s="59" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="64"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="64"/>
-      <c r="J10" s="64"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
       <c r="K10" s="60"/>
     </row>
     <row r="11" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F11" s="65" t="s">
+      <c r="F11" s="62" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="66"/>
-      <c r="H11" s="66"/>
-      <c r="I11" s="67"/>
-      <c r="J11" s="56" t="s">
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="64"/>
+      <c r="J11" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="K11" s="56"/>
+      <c r="K11" s="66"/>
     </row>
     <row r="12" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F12" s="57" t="s">
+      <c r="F12" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
-      <c r="I12" s="57"/>
-      <c r="J12" s="56">
-        <v>0</v>
-      </c>
-      <c r="K12" s="56"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="66">
+        <v>0</v>
+      </c>
+      <c r="K12" s="66"/>
     </row>
     <row r="13" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F13" s="57" t="s">
+      <c r="F13" s="65" t="s">
         <v>71</v>
       </c>
-      <c r="G13" s="57"/>
-      <c r="H13" s="57"/>
-      <c r="I13" s="57"/>
-      <c r="J13" s="56">
-        <v>0</v>
-      </c>
-      <c r="K13" s="56"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="65"/>
+      <c r="I13" s="65"/>
+      <c r="J13" s="66">
+        <v>0</v>
+      </c>
+      <c r="K13" s="66"/>
     </row>
     <row r="14" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="56">
-        <v>0</v>
-      </c>
-      <c r="K14" s="56"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="66">
+        <v>0</v>
+      </c>
+      <c r="K14" s="66"/>
     </row>
     <row r="15" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F15" s="57" t="s">
+      <c r="F15" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="G15" s="57"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="56">
-        <v>0</v>
-      </c>
-      <c r="K15" s="56"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
+      <c r="I15" s="65"/>
+      <c r="J15" s="66">
+        <v>0</v>
+      </c>
+      <c r="K15" s="66"/>
     </row>
     <row r="16" spans="6:19" x14ac:dyDescent="0.25">
-      <c r="F16" s="57" t="s">
+      <c r="F16" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="56">
-        <v>0</v>
-      </c>
-      <c r="K16" s="56"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
+      <c r="I16" s="65"/>
+      <c r="J16" s="66">
+        <v>0</v>
+      </c>
+      <c r="K16" s="66"/>
     </row>
     <row r="17" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F17" s="61" t="s">
+      <c r="F17" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="63"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="58"/>
       <c r="J17" s="59">
         <v>0</v>
       </c>
       <c r="K17" s="60"/>
     </row>
     <row r="18" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F18" s="57" t="s">
+      <c r="F18" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="57"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="56">
-        <v>0</v>
-      </c>
-      <c r="K18" s="56"/>
+      <c r="G18" s="65"/>
+      <c r="H18" s="65"/>
+      <c r="I18" s="65"/>
+      <c r="J18" s="66">
+        <v>0</v>
+      </c>
+      <c r="K18" s="66"/>
     </row>
     <row r="19" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="63"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="58"/>
       <c r="J19" s="59">
         <v>0</v>
       </c>
       <c r="K19" s="60"/>
     </row>
     <row r="20" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F20" s="61"/>
-      <c r="G20" s="62"/>
-      <c r="H20" s="62"/>
-      <c r="I20" s="63"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="57"/>
+      <c r="I20" s="58"/>
       <c r="J20" s="59"/>
       <c r="K20" s="60"/>
     </row>
     <row r="21" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F21" s="61"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="63"/>
+      <c r="F21" s="56"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57"/>
+      <c r="I21" s="58"/>
       <c r="J21" s="59"/>
       <c r="K21" s="60"/>
     </row>
     <row r="22" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F22" s="58"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="58"/>
-      <c r="I22" s="58"/>
-      <c r="J22" s="56"/>
-      <c r="K22" s="56"/>
+      <c r="F22" s="68"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="66"/>
+      <c r="K22" s="66"/>
     </row>
     <row r="23" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="F23" s="56" t="s">
+      <c r="F23" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="56">
+      <c r="G23" s="66"/>
+      <c r="H23" s="66"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="66">
         <f>SUM(J12:K22)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="56"/>
+      <c r="K23" s="66"/>
     </row>
     <row r="27" spans="6:15" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
@@ -8173,12 +8178,12 @@
       </c>
     </row>
     <row r="29" spans="6:15" x14ac:dyDescent="0.25">
-      <c r="J29" s="40" t="s">
+      <c r="J29" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="K29" s="55"/>
-      <c r="L29" s="55"/>
-      <c r="M29" s="55"/>
+      <c r="K29" s="67"/>
+      <c r="L29" s="67"/>
+      <c r="M29" s="67"/>
     </row>
     <row r="31" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O31" t="s">
@@ -8187,6 +8192,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F21:I21"/>
     <mergeCell ref="F20:I20"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="J21:K21"/>
@@ -8203,22 +8224,6 @@
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F21:I21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8246,85 +8251,85 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="37"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C6" s="68" t="s">
+      <c r="C6" s="76" t="s">
         <v>133</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B9" s="14" t="s">
@@ -8333,18 +8338,18 @@
       <c r="C9" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="69" t="s">
+      <c r="D9" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="E9" s="69"/>
-      <c r="F9" s="70" t="s">
+      <c r="E9" s="75"/>
+      <c r="F9" s="71" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="70"/>
-      <c r="H9" s="70" t="s">
+      <c r="G9" s="71"/>
+      <c r="H9" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="70"/>
+      <c r="I9" s="71"/>
       <c r="J9" s="72" t="s">
         <v>53</v>
       </c>
@@ -8354,472 +8359,472 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="42" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="70">
-        <v>0</v>
-      </c>
-      <c r="E10" s="70"/>
-      <c r="F10" s="71">
-        <v>0</v>
-      </c>
-      <c r="G10" s="71"/>
-      <c r="H10" s="70">
-        <v>0</v>
-      </c>
-      <c r="I10" s="70"/>
-      <c r="J10" s="74">
-        <v>0</v>
-      </c>
-      <c r="K10" s="75"/>
+      <c r="D10" s="71">
+        <v>0</v>
+      </c>
+      <c r="E10" s="71"/>
+      <c r="F10" s="74">
+        <v>0</v>
+      </c>
+      <c r="G10" s="74"/>
+      <c r="H10" s="71">
+        <v>0</v>
+      </c>
+      <c r="I10" s="71"/>
+      <c r="J10" s="69">
+        <v>0</v>
+      </c>
+      <c r="K10" s="70"/>
       <c r="L10" s="2">
         <f t="shared" ref="L10:L17" si="0">SUM(D10:K10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="42"/>
+      <c r="B11" s="43"/>
       <c r="C11" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="70">
-        <v>0</v>
-      </c>
-      <c r="E11" s="70"/>
-      <c r="F11" s="71">
-        <v>0</v>
-      </c>
-      <c r="G11" s="71"/>
-      <c r="H11" s="70">
-        <v>0</v>
-      </c>
-      <c r="I11" s="70"/>
-      <c r="J11" s="74">
-        <v>0</v>
-      </c>
-      <c r="K11" s="75"/>
+      <c r="D11" s="71">
+        <v>0</v>
+      </c>
+      <c r="E11" s="71"/>
+      <c r="F11" s="74">
+        <v>0</v>
+      </c>
+      <c r="G11" s="74"/>
+      <c r="H11" s="71">
+        <v>0</v>
+      </c>
+      <c r="I11" s="71"/>
+      <c r="J11" s="69">
+        <v>0</v>
+      </c>
+      <c r="K11" s="70"/>
       <c r="L11" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="42"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="70">
-        <v>0</v>
-      </c>
-      <c r="E12" s="70"/>
-      <c r="F12" s="71">
-        <v>0</v>
-      </c>
-      <c r="G12" s="71"/>
-      <c r="H12" s="70">
-        <v>0</v>
-      </c>
-      <c r="I12" s="70"/>
-      <c r="J12" s="74">
-        <v>0</v>
-      </c>
-      <c r="K12" s="75"/>
+      <c r="D12" s="71">
+        <v>0</v>
+      </c>
+      <c r="E12" s="71"/>
+      <c r="F12" s="74">
+        <v>0</v>
+      </c>
+      <c r="G12" s="74"/>
+      <c r="H12" s="71">
+        <v>0</v>
+      </c>
+      <c r="I12" s="71"/>
+      <c r="J12" s="69">
+        <v>0</v>
+      </c>
+      <c r="K12" s="70"/>
       <c r="L12" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="42"/>
+      <c r="B13" s="43"/>
       <c r="C13" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="70">
-        <v>0</v>
-      </c>
-      <c r="E13" s="70"/>
-      <c r="F13" s="71">
-        <v>0</v>
-      </c>
-      <c r="G13" s="71"/>
-      <c r="H13" s="70">
-        <v>0</v>
-      </c>
-      <c r="I13" s="70"/>
-      <c r="J13" s="74">
-        <v>0</v>
-      </c>
-      <c r="K13" s="75"/>
+      <c r="D13" s="71">
+        <v>0</v>
+      </c>
+      <c r="E13" s="71"/>
+      <c r="F13" s="74">
+        <v>0</v>
+      </c>
+      <c r="G13" s="74"/>
+      <c r="H13" s="71">
+        <v>0</v>
+      </c>
+      <c r="I13" s="71"/>
+      <c r="J13" s="69">
+        <v>0</v>
+      </c>
+      <c r="K13" s="70"/>
       <c r="L13" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="42"/>
+      <c r="B14" s="43"/>
       <c r="C14" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="70">
-        <v>0</v>
-      </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="71">
-        <v>0</v>
-      </c>
-      <c r="G14" s="71"/>
-      <c r="H14" s="70">
-        <v>0</v>
-      </c>
-      <c r="I14" s="70"/>
-      <c r="J14" s="74">
-        <v>0</v>
-      </c>
-      <c r="K14" s="75"/>
+      <c r="D14" s="71">
+        <v>0</v>
+      </c>
+      <c r="E14" s="71"/>
+      <c r="F14" s="74">
+        <v>0</v>
+      </c>
+      <c r="G14" s="74"/>
+      <c r="H14" s="71">
+        <v>0</v>
+      </c>
+      <c r="I14" s="71"/>
+      <c r="J14" s="69">
+        <v>0</v>
+      </c>
+      <c r="K14" s="70"/>
       <c r="L14" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B15" s="42"/>
+      <c r="B15" s="43"/>
       <c r="C15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="70">
-        <v>0</v>
-      </c>
-      <c r="E15" s="70"/>
-      <c r="F15" s="71">
-        <v>0</v>
-      </c>
-      <c r="G15" s="71"/>
-      <c r="H15" s="70">
-        <v>0</v>
-      </c>
-      <c r="I15" s="70"/>
-      <c r="J15" s="74">
-        <v>0</v>
-      </c>
-      <c r="K15" s="75"/>
+      <c r="D15" s="71">
+        <v>0</v>
+      </c>
+      <c r="E15" s="71"/>
+      <c r="F15" s="74">
+        <v>0</v>
+      </c>
+      <c r="G15" s="74"/>
+      <c r="H15" s="71">
+        <v>0</v>
+      </c>
+      <c r="I15" s="71"/>
+      <c r="J15" s="69">
+        <v>0</v>
+      </c>
+      <c r="K15" s="70"/>
       <c r="L15" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="42"/>
+      <c r="B16" s="43"/>
       <c r="C16" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="70">
-        <v>0</v>
-      </c>
-      <c r="E16" s="70"/>
-      <c r="F16" s="71">
-        <v>0</v>
-      </c>
-      <c r="G16" s="71"/>
-      <c r="H16" s="70">
-        <v>0</v>
-      </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="74">
-        <v>0</v>
-      </c>
-      <c r="K16" s="75"/>
+      <c r="D16" s="71">
+        <v>0</v>
+      </c>
+      <c r="E16" s="71"/>
+      <c r="F16" s="74">
+        <v>0</v>
+      </c>
+      <c r="G16" s="74"/>
+      <c r="H16" s="71">
+        <v>0</v>
+      </c>
+      <c r="I16" s="71"/>
+      <c r="J16" s="69">
+        <v>0</v>
+      </c>
+      <c r="K16" s="70"/>
       <c r="L16" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="42"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="70">
-        <v>0</v>
-      </c>
-      <c r="E17" s="70"/>
-      <c r="F17" s="71">
-        <v>0</v>
-      </c>
-      <c r="G17" s="71"/>
-      <c r="H17" s="70">
-        <v>0</v>
-      </c>
-      <c r="I17" s="70"/>
-      <c r="J17" s="74">
-        <v>0</v>
-      </c>
-      <c r="K17" s="75"/>
+      <c r="D17" s="71">
+        <v>0</v>
+      </c>
+      <c r="E17" s="71"/>
+      <c r="F17" s="74">
+        <v>0</v>
+      </c>
+      <c r="G17" s="74"/>
+      <c r="H17" s="71">
+        <v>0</v>
+      </c>
+      <c r="I17" s="71"/>
+      <c r="J17" s="69">
+        <v>0</v>
+      </c>
+      <c r="K17" s="70"/>
       <c r="L17" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="70">
-        <v>0</v>
-      </c>
-      <c r="E18" s="70"/>
-      <c r="F18" s="71">
-        <v>0</v>
-      </c>
-      <c r="G18" s="71"/>
-      <c r="H18" s="70">
-        <v>0</v>
-      </c>
-      <c r="I18" s="70"/>
-      <c r="J18" s="74">
-        <v>0</v>
-      </c>
-      <c r="K18" s="75"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="71">
+        <v>0</v>
+      </c>
+      <c r="E18" s="71"/>
+      <c r="F18" s="74">
+        <v>0</v>
+      </c>
+      <c r="G18" s="74"/>
+      <c r="H18" s="71">
+        <v>0</v>
+      </c>
+      <c r="I18" s="71"/>
+      <c r="J18" s="69">
+        <v>0</v>
+      </c>
+      <c r="K18" s="70"/>
       <c r="L18" s="2">
         <f>SUM(L10:L17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="48" t="s">
         <v>34</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="70">
-        <v>0</v>
-      </c>
-      <c r="E19" s="70"/>
-      <c r="F19" s="71">
-        <v>0</v>
-      </c>
-      <c r="G19" s="71"/>
-      <c r="H19" s="70">
-        <v>0</v>
-      </c>
-      <c r="I19" s="70"/>
-      <c r="J19" s="74">
-        <v>0</v>
-      </c>
-      <c r="K19" s="75"/>
+      <c r="D19" s="71">
+        <v>0</v>
+      </c>
+      <c r="E19" s="71"/>
+      <c r="F19" s="74">
+        <v>0</v>
+      </c>
+      <c r="G19" s="74"/>
+      <c r="H19" s="71">
+        <v>0</v>
+      </c>
+      <c r="I19" s="71"/>
+      <c r="J19" s="69">
+        <v>0</v>
+      </c>
+      <c r="K19" s="70"/>
       <c r="L19" s="2">
         <f t="shared" ref="L19:L26" si="1">SUM(D19:K19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="48"/>
+      <c r="B20" s="49"/>
       <c r="C20" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="70">
-        <v>0</v>
-      </c>
-      <c r="E20" s="70"/>
-      <c r="F20" s="71">
-        <v>0</v>
-      </c>
-      <c r="G20" s="71"/>
-      <c r="H20" s="70">
-        <v>0</v>
-      </c>
-      <c r="I20" s="70"/>
-      <c r="J20" s="74">
-        <v>0</v>
-      </c>
-      <c r="K20" s="75"/>
+      <c r="D20" s="71">
+        <v>0</v>
+      </c>
+      <c r="E20" s="71"/>
+      <c r="F20" s="74">
+        <v>0</v>
+      </c>
+      <c r="G20" s="74"/>
+      <c r="H20" s="71">
+        <v>0</v>
+      </c>
+      <c r="I20" s="71"/>
+      <c r="J20" s="69">
+        <v>0</v>
+      </c>
+      <c r="K20" s="70"/>
       <c r="L20" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="48"/>
+      <c r="B21" s="49"/>
       <c r="C21" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="70">
-        <v>0</v>
-      </c>
-      <c r="E21" s="70"/>
-      <c r="F21" s="71">
-        <v>0</v>
-      </c>
-      <c r="G21" s="71"/>
-      <c r="H21" s="70">
-        <v>0</v>
-      </c>
-      <c r="I21" s="70"/>
-      <c r="J21" s="74">
-        <v>0</v>
-      </c>
-      <c r="K21" s="75"/>
+      <c r="D21" s="71">
+        <v>0</v>
+      </c>
+      <c r="E21" s="71"/>
+      <c r="F21" s="74">
+        <v>0</v>
+      </c>
+      <c r="G21" s="74"/>
+      <c r="H21" s="71">
+        <v>0</v>
+      </c>
+      <c r="I21" s="71"/>
+      <c r="J21" s="69">
+        <v>0</v>
+      </c>
+      <c r="K21" s="70"/>
       <c r="L21" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="48"/>
+      <c r="B22" s="49"/>
       <c r="C22" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="70">
-        <v>0</v>
-      </c>
-      <c r="E22" s="70"/>
-      <c r="F22" s="71">
-        <v>0</v>
-      </c>
-      <c r="G22" s="71"/>
-      <c r="H22" s="70">
-        <v>0</v>
-      </c>
-      <c r="I22" s="70"/>
-      <c r="J22" s="74">
-        <v>0</v>
-      </c>
-      <c r="K22" s="75"/>
+      <c r="D22" s="71">
+        <v>0</v>
+      </c>
+      <c r="E22" s="71"/>
+      <c r="F22" s="74">
+        <v>0</v>
+      </c>
+      <c r="G22" s="74"/>
+      <c r="H22" s="71">
+        <v>0</v>
+      </c>
+      <c r="I22" s="71"/>
+      <c r="J22" s="69">
+        <v>0</v>
+      </c>
+      <c r="K22" s="70"/>
       <c r="L22" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B23" s="48"/>
+      <c r="B23" s="49"/>
       <c r="C23" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="70">
-        <v>0</v>
-      </c>
-      <c r="E23" s="70"/>
-      <c r="F23" s="71">
-        <v>0</v>
-      </c>
-      <c r="G23" s="71"/>
-      <c r="H23" s="70">
-        <v>0</v>
-      </c>
-      <c r="I23" s="70"/>
-      <c r="J23" s="74">
-        <v>0</v>
-      </c>
-      <c r="K23" s="75"/>
+      <c r="D23" s="71">
+        <v>0</v>
+      </c>
+      <c r="E23" s="71"/>
+      <c r="F23" s="74">
+        <v>0</v>
+      </c>
+      <c r="G23" s="74"/>
+      <c r="H23" s="71">
+        <v>0</v>
+      </c>
+      <c r="I23" s="71"/>
+      <c r="J23" s="69">
+        <v>0</v>
+      </c>
+      <c r="K23" s="70"/>
       <c r="L23" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="48"/>
+      <c r="B24" s="49"/>
       <c r="C24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="70">
-        <v>0</v>
-      </c>
-      <c r="E24" s="70"/>
-      <c r="F24" s="71">
-        <v>0</v>
-      </c>
-      <c r="G24" s="71"/>
-      <c r="H24" s="70">
-        <v>0</v>
-      </c>
-      <c r="I24" s="70"/>
-      <c r="J24" s="74">
-        <v>0</v>
-      </c>
-      <c r="K24" s="75"/>
+      <c r="D24" s="71">
+        <v>0</v>
+      </c>
+      <c r="E24" s="71"/>
+      <c r="F24" s="74">
+        <v>0</v>
+      </c>
+      <c r="G24" s="74"/>
+      <c r="H24" s="71">
+        <v>0</v>
+      </c>
+      <c r="I24" s="71"/>
+      <c r="J24" s="69">
+        <v>0</v>
+      </c>
+      <c r="K24" s="70"/>
       <c r="L24" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="48"/>
+      <c r="B25" s="49"/>
       <c r="C25" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="70">
-        <v>0</v>
-      </c>
-      <c r="E25" s="70"/>
-      <c r="F25" s="71">
-        <v>0</v>
-      </c>
-      <c r="G25" s="71"/>
-      <c r="H25" s="70">
-        <v>0</v>
-      </c>
-      <c r="I25" s="70"/>
-      <c r="J25" s="74">
-        <v>0</v>
-      </c>
-      <c r="K25" s="75"/>
+      <c r="D25" s="71">
+        <v>0</v>
+      </c>
+      <c r="E25" s="71"/>
+      <c r="F25" s="74">
+        <v>0</v>
+      </c>
+      <c r="G25" s="74"/>
+      <c r="H25" s="71">
+        <v>0</v>
+      </c>
+      <c r="I25" s="71"/>
+      <c r="J25" s="69">
+        <v>0</v>
+      </c>
+      <c r="K25" s="70"/>
       <c r="L25" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="49"/>
+      <c r="B26" s="50"/>
       <c r="C26" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="70">
-        <v>0</v>
-      </c>
-      <c r="E26" s="70"/>
-      <c r="F26" s="71">
-        <v>0</v>
-      </c>
-      <c r="G26" s="71"/>
-      <c r="H26" s="70">
-        <v>0</v>
-      </c>
-      <c r="I26" s="70"/>
-      <c r="J26" s="74">
-        <v>0</v>
-      </c>
-      <c r="K26" s="75"/>
+      <c r="D26" s="71">
+        <v>0</v>
+      </c>
+      <c r="E26" s="71"/>
+      <c r="F26" s="74">
+        <v>0</v>
+      </c>
+      <c r="G26" s="74"/>
+      <c r="H26" s="71">
+        <v>0</v>
+      </c>
+      <c r="I26" s="71"/>
+      <c r="J26" s="69">
+        <v>0</v>
+      </c>
+      <c r="K26" s="70"/>
       <c r="L26" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="70">
-        <v>0</v>
-      </c>
-      <c r="E27" s="70"/>
-      <c r="F27" s="71">
-        <v>0</v>
-      </c>
-      <c r="G27" s="71"/>
-      <c r="H27" s="70">
-        <v>0</v>
-      </c>
-      <c r="I27" s="70"/>
-      <c r="J27" s="74">
-        <v>0</v>
-      </c>
-      <c r="K27" s="75"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="71">
+        <v>0</v>
+      </c>
+      <c r="E27" s="71"/>
+      <c r="F27" s="74">
+        <v>0</v>
+      </c>
+      <c r="G27" s="74"/>
+      <c r="H27" s="71">
+        <v>0</v>
+      </c>
+      <c r="I27" s="71"/>
+      <c r="J27" s="69">
+        <v>0</v>
+      </c>
+      <c r="K27" s="70"/>
       <c r="L27" s="2">
         <f>SUM(L19:L26)</f>
         <v>0</v>
@@ -8836,12 +8841,12 @@
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="I31" s="40" t="s">
+      <c r="I31" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="40"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
     </row>
     <row r="33" spans="12:12" x14ac:dyDescent="0.25">
       <c r="L33" t="s">
@@ -8850,16 +8855,66 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:B26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B10:B17"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="J10:K10"/>
@@ -8876,66 +8931,16 @@
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="H26:I26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:B26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B10:B17"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8955,13 +8960,13 @@
   </cols>
   <sheetData>
     <row r="3" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E3" s="36" t="s">
+      <c r="E3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
       <c r="J3" s="18"/>
       <c r="K3" s="18"/>
       <c r="L3" s="18"/>
@@ -8974,14 +8979,14 @@
       <c r="S3" s="18"/>
     </row>
     <row r="4" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
@@ -8993,14 +8998,14 @@
       <c r="S4" s="18"/>
     </row>
     <row r="5" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E5" s="36" t="s">
+      <c r="E5" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -9012,14 +9017,14 @@
       <c r="S5" s="18"/>
     </row>
     <row r="6" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
       <c r="K6" s="19"/>
       <c r="L6" s="19"/>
       <c r="M6" s="19"/>
@@ -9031,176 +9036,176 @@
       <c r="S6" s="19"/>
     </row>
     <row r="7" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E7" s="34" t="s">
+      <c r="E7" s="28" t="s">
         <v>134</v>
       </c>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="34"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
     </row>
     <row r="9" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E9" s="70" t="s">
+      <c r="E9" s="71" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="70"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="70"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="70"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
+      <c r="I9" s="71"/>
+      <c r="J9" s="71"/>
     </row>
     <row r="10" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E10" s="76" t="s">
+      <c r="E10" s="77" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="56">
-        <v>0</v>
-      </c>
-      <c r="J10" s="56"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="66">
+        <v>0</v>
+      </c>
+      <c r="J10" s="66"/>
     </row>
     <row r="11" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E11" s="76" t="s">
+      <c r="E11" s="77" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
-      <c r="I11" s="56">
-        <v>0</v>
-      </c>
-      <c r="J11" s="56"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="66">
+        <v>0</v>
+      </c>
+      <c r="J11" s="66"/>
     </row>
     <row r="12" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E12" s="76" t="s">
+      <c r="E12" s="77" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
-      <c r="I12" s="56">
-        <v>0</v>
-      </c>
-      <c r="J12" s="56"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="66">
+        <v>0</v>
+      </c>
+      <c r="J12" s="66"/>
     </row>
     <row r="13" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E13" s="76" t="s">
+      <c r="E13" s="77" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="76"/>
-      <c r="G13" s="76"/>
-      <c r="H13" s="76"/>
-      <c r="I13" s="56">
-        <v>0</v>
-      </c>
-      <c r="J13" s="56"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="66">
+        <v>0</v>
+      </c>
+      <c r="J13" s="66"/>
     </row>
     <row r="14" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E14" s="76" t="s">
+      <c r="E14" s="77" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="76"/>
-      <c r="G14" s="76"/>
-      <c r="H14" s="76"/>
-      <c r="I14" s="56">
-        <v>0</v>
-      </c>
-      <c r="J14" s="56"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="66">
+        <v>0</v>
+      </c>
+      <c r="J14" s="66"/>
     </row>
     <row r="15" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E15" s="76" t="s">
+      <c r="E15" s="77" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
-      <c r="I15" s="56">
-        <v>0</v>
-      </c>
-      <c r="J15" s="56"/>
+      <c r="F15" s="77"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="77"/>
+      <c r="I15" s="66">
+        <v>0</v>
+      </c>
+      <c r="J15" s="66"/>
     </row>
     <row r="16" spans="5:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E16" s="77" t="s">
+      <c r="E16" s="78" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="56">
-        <v>0</v>
-      </c>
-      <c r="J16" s="56"/>
+      <c r="F16" s="78"/>
+      <c r="G16" s="78"/>
+      <c r="H16" s="78"/>
+      <c r="I16" s="66">
+        <v>0</v>
+      </c>
+      <c r="J16" s="66"/>
     </row>
     <row r="17" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E17" s="76" t="s">
+      <c r="E17" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="76"/>
-      <c r="G17" s="76"/>
-      <c r="H17" s="76"/>
-      <c r="I17" s="56">
-        <v>0</v>
-      </c>
-      <c r="J17" s="56"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="66">
+        <v>0</v>
+      </c>
+      <c r="J17" s="66"/>
     </row>
     <row r="18" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E18" s="76" t="s">
+      <c r="E18" s="77" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="76"/>
-      <c r="I18" s="56">
-        <v>0</v>
-      </c>
-      <c r="J18" s="56"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="66">
+        <v>0</v>
+      </c>
+      <c r="J18" s="66"/>
     </row>
     <row r="19" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E19" s="78" t="s">
+      <c r="E19" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="79"/>
-      <c r="G19" s="79"/>
-      <c r="H19" s="80"/>
+      <c r="F19" s="80"/>
+      <c r="G19" s="80"/>
+      <c r="H19" s="81"/>
       <c r="I19" s="59">
         <v>0</v>
       </c>
       <c r="J19" s="60"/>
     </row>
     <row r="20" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E20" s="76" t="s">
+      <c r="E20" s="77" t="s">
         <v>64</v>
       </c>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="76"/>
-      <c r="I20" s="56">
-        <v>0</v>
-      </c>
-      <c r="J20" s="56"/>
+      <c r="F20" s="77"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="66">
+        <v>0</v>
+      </c>
+      <c r="J20" s="66"/>
     </row>
     <row r="21" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E21" s="81" t="s">
+      <c r="E21" s="82" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="84"/>
       <c r="I21" s="59">
         <v>0</v>
       </c>
       <c r="J21" s="60"/>
     </row>
     <row r="22" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E22" s="78" t="s">
+      <c r="E22" s="79" t="s">
         <v>80</v>
       </c>
-      <c r="F22" s="79"/>
-      <c r="G22" s="79"/>
-      <c r="H22" s="80"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="80"/>
+      <c r="H22" s="81"/>
       <c r="I22" s="59">
         <f>SUM(I20:J21)</f>
         <v>0</v>
@@ -9208,41 +9213,41 @@
       <c r="J22" s="60"/>
     </row>
     <row r="23" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E23" s="76" t="s">
+      <c r="E23" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="76"/>
-      <c r="I23" s="56">
-        <v>0</v>
-      </c>
-      <c r="J23" s="56"/>
+      <c r="F23" s="77"/>
+      <c r="G23" s="77"/>
+      <c r="H23" s="77"/>
+      <c r="I23" s="66">
+        <v>0</v>
+      </c>
+      <c r="J23" s="66"/>
     </row>
     <row r="24" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E24" s="76" t="s">
+      <c r="E24" s="77" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="76"/>
-      <c r="I24" s="56">
-        <v>0</v>
-      </c>
-      <c r="J24" s="56"/>
+      <c r="F24" s="77"/>
+      <c r="G24" s="77"/>
+      <c r="H24" s="77"/>
+      <c r="I24" s="66">
+        <v>0</v>
+      </c>
+      <c r="J24" s="66"/>
     </row>
     <row r="25" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E25" s="77" t="s">
+      <c r="E25" s="78" t="s">
         <v>81</v>
       </c>
-      <c r="F25" s="77"/>
-      <c r="G25" s="77"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="56">
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
+      <c r="I25" s="66">
         <f>SUM(I23:J24)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="56"/>
+      <c r="J25" s="66"/>
     </row>
     <row r="28" spans="5:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="H28" t="s">
@@ -9270,6 +9275,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="E7:J7"/>
+    <mergeCell ref="E9:J9"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I19:J19"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="E24:H24"/>
     <mergeCell ref="E25:H25"/>
@@ -9286,28 +9313,6 @@
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="E7:J7"/>
-    <mergeCell ref="E9:J9"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>

</xml_diff>